<commit_message>
Mise à jour de l'appel au VS des sections suite au création du JDV sur le SMT 0d4ad507382de183999fbbaca99928f80640c73f
</commit_message>
<xml_diff>
--- a/SectionsFHIRCorps/ig/StructureDefinition-fr-composition-document.xlsx
+++ b/SectionsFHIRCorps/ig/StructureDefinition-fr-composition-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-04T08:48:36+00:00</t>
+    <t>2026-03-12T10:53:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2573,7 +2573,7 @@
     <t>Provides computable standardized labels to topics within the document.</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/ValueSet/fr-vs-liste-sections</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-section-document-cisis</t>
   </si>
   <si>
     <t>Composition.section.author</t>
@@ -32276,7 +32276,7 @@
         <v>78</v>
       </c>
       <c r="X251" t="s" s="2">
-        <v>153</v>
+        <v>323</v>
       </c>
       <c r="Y251" s="2"/>
       <c r="Z251" t="s" s="2">

</xml_diff>